<commit_message>
before the color change
</commit_message>
<xml_diff>
--- a/src/spreadsheets/shippingCredentials.xlsx
+++ b/src/spreadsheets/shippingCredentials.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="25">
   <si>
     <t>John Doe Mária</t>
   </si>
@@ -80,6 +80,15 @@
   </si>
   <si>
     <t>forpeoplpe13@gmail.com</t>
+  </si>
+  <si>
+    <t>asd</t>
+  </si>
+  <si>
+    <t>0797447899</t>
+  </si>
+  <si>
+    <t>Parts</t>
   </si>
 </sst>
 </file>
@@ -1340,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:N128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.83333"/>
   <cols>
     <col min="1" max="1" width="16.1719" style="1" customWidth="1"/>
@@ -4917,6 +4926,47 @@
         <v>36792</v>
       </c>
     </row>
+    <row r="128" ht="13.55" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A128" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C128" s="1">
+        <v>0</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G128" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I128" s="1">
+        <v>15</v>
+      </c>
+      <c r="J128" s="1">
+        <v>20</v>
+      </c>
+      <c r="K128" s="1">
+        <v>15</v>
+      </c>
+      <c r="L128" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M128" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N128" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>